<commit_message>
docs(demos): cierra gaps de la auditoría — entrega de cuenta, instituciones nombradas, caveat de IA
- Nuevo correo-entrega-cuenta-docente.md: mensaje (correo + WhatsApp) que ENTREGA la
  cuenta con URL, "elige ExamLab Demo", usuario+contraseña, video de login y primeros pasos.
- Manual ("Cómo ingresar") + manual-docente: nombran la institución "ExamLab Demo",
  avisan que el tenant viene vacío (crear curso, sin estudiantes) y aclaran que los
  paths de video son del repo (no enlaces).
- Excel: columna Notas con la advertencia de tenant vacío + contraseña genérica.
- Caveat añadido en manual, manual-docente, Excel y correo de entrega: si la IA falla
  en el demo suele ser disponibilidad del modelo — reintentar, no es un bug.
- WhatsApp: testimonios en 1ª persona condicionados a "solo si ya lo probaste";
  corregida la referencia cruzada engañosa; paridad de links (Excel + video login).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demos/correos/ExamLab-Usuarios-Demo.xlsx
+++ b/docs/demos/correos/ExamLab-Usuarios-Demo.xlsx
@@ -112,7 +112,11 @@
       </c>
       <c r="H2"/>
       <c r="I2"/>
-      <c r="J2"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -152,7 +156,11 @@
       </c>
       <c r="H3"/>
       <c r="I3"/>
-      <c r="J3"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -192,7 +200,11 @@
       </c>
       <c r="H4"/>
       <c r="I4"/>
-      <c r="J4"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -232,7 +244,11 @@
       </c>
       <c r="H5"/>
       <c r="I5"/>
-      <c r="J5"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -272,7 +288,11 @@
       </c>
       <c r="H6"/>
       <c r="I6"/>
-      <c r="J6"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
docs(demos): refleja el doble rol Docente+Estudiante en mensajes, Excel y manual
Las 5 cuentas demo ahora tienen rol Docente Y Estudiante (cambio aplicado en DB).
Se comunica en lo que recibe el docente para que sepa qué hacer:
- correo-entrega + correo-colegas: nota "tienes dos roles, cámbialos con el selector".
- Excel: columna Rol = "Docente + Estudiante" + nota de cambio de rol.
- manual.md / manual-docente.md: nota de doble rol en el bloque de cuenta demo.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demos/correos/ExamLab-Usuarios-Demo.xlsx
+++ b/docs/demos/correos/ExamLab-Usuarios-Demo.xlsx
@@ -97,7 +97,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Docente</t>
+          <t xml:space="preserve">Docente + Estudiante</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -114,7 +114,7 @@
       <c r="I2"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma.</t>
+          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma. La cuenta tiene dos roles (Docente y Estudiante): cambia con el selector arriba del menú para ver ambas vistas.</t>
         </is>
       </c>
     </row>
@@ -141,7 +141,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Docente</t>
+          <t xml:space="preserve">Docente + Estudiante</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -158,7 +158,7 @@
       <c r="I3"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma.</t>
+          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma. La cuenta tiene dos roles (Docente y Estudiante): cambia con el selector arriba del menú para ver ambas vistas.</t>
         </is>
       </c>
     </row>
@@ -185,7 +185,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Docente</t>
+          <t xml:space="preserve">Docente + Estudiante</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -202,7 +202,7 @@
       <c r="I4"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma.</t>
+          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma. La cuenta tiene dos roles (Docente y Estudiante): cambia con el selector arriba del menú para ver ambas vistas.</t>
         </is>
       </c>
     </row>
@@ -229,7 +229,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Docente</t>
+          <t xml:space="preserve">Docente + Estudiante</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -246,7 +246,7 @@
       <c r="I5"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma.</t>
+          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma. La cuenta tiene dos roles (Docente y Estudiante): cambia con el selector arriba del menú para ver ambas vistas.</t>
         </is>
       </c>
     </row>
@@ -273,7 +273,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Docente</t>
+          <t xml:space="preserve">Docente + Estudiante</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -290,7 +290,7 @@
       <c r="I6"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma.</t>
+          <t xml:space="preserve">Cuenta de demo. Al iniciar sesión, selecciona la institución "ExamLab Demo". El espacio empieza vacío: crea tu propio curso para empezar y usa la IA para generar exámenes/talleres (corre al instante). No incluye estudiantes (la matrícula la hace un administrador), así que el ciclo completo de calificación de entregas reales se ve en los videos demo, no en esta cuenta. La contraseña es genérica y no caduca al primer ingreso. Si la IA falla puntualmente, suele ser disponibilidad del modelo (es una demo): espera unos minutos y reintenta — no es un error de la plataforma. La cuenta tiene dos roles (Docente y Estudiante): cambia con el selector arriba del menú para ver ambas vistas.</t>
         </is>
       </c>
     </row>

</xml_diff>